<commit_message>
feat: add scripts for PDF hour auditing and Jira project reporting tools
</commit_message>
<xml_diff>
--- a/refs/planilhas/RevisaoForms.xlsx
+++ b/refs/planilhas/RevisaoForms.xlsx
@@ -28,13 +28,13 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={2b894185-2081-4d23-aa1b-4055f8e1f2a8}</author>
-    <author>tc={99afa052-999d-44e4-8770-211425b04150}</author>
-    <author>tc={da57aa93-8abe-4959-84c8-4bf38f451ac0}</author>
-    <author>tc={f5a66fda-0c81-42df-af30-4c66e2255bc0}</author>
+    <author>tc={106fe65b-207a-4fef-bb5d-65c426ae0dfe}</author>
+    <author>tc={3e2ffa88-8395-46b4-a6ff-8043f985b458}</author>
+    <author>tc={9310f6d9-ace3-4304-81fe-60292bb798e5}</author>
+    <author>tc={cada2db6-c675-4d37-b110-ba5b0f389f52}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{2b894185-2081-4d23-aa1b-4055f8e1f2a8}" ref="A35">
+    <comment authorId="0" xr:uid="{106fe65b-207a-4fef-bb5d-65c426ae0dfe}" ref="A35">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -43,7 +43,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{99afa052-999d-44e4-8770-211425b04150}" ref="A18">
+    <comment authorId="1" xr:uid="{3e2ffa88-8395-46b4-a6ff-8043f985b458}" ref="A18">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -52,7 +52,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{da57aa93-8abe-4959-84c8-4bf38f451ac0}" ref="A26">
+    <comment authorId="2" xr:uid="{9310f6d9-ace3-4304-81fe-60292bb798e5}" ref="A26">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -61,7 +61,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{f5a66fda-0c81-42df-af30-4c66e2255bc0}" ref="A18">
+    <comment authorId="3" xr:uid="{cada2db6-c675-4d37-b110-ba5b0f389f52}" ref="A18">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -77,10 +77,10 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={4e9f8ac5-f033-44ea-b9dc-147610cecf1c}</author>
+    <author>tc={748f1715-cd33-4762-9a80-024903a734da}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{4e9f8ac5-f033-44ea-b9dc-147610cecf1c}" ref="A3">
+    <comment authorId="0" xr:uid="{748f1715-cd33-4762-9a80-024903a734da}" ref="A3">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1748" uniqueCount="224">
   <si>
     <t>OBSERVAÇÕES GERAIS</t>
   </si>
@@ -722,13 +722,10 @@
     <t>Atividades exercidas no local:</t>
   </si>
   <si>
-    <t>Orgao muda atuação em fç da atividade? ex camelo leva apenas moto, feira leva caminhao p recolher tudo</t>
-  </si>
-  <si>
     <t>Indicação da área ocupada:</t>
   </si>
   <si>
-    <t>É importante pro orgão saber essa informação?o que isso muda na atuação dele</t>
+    <t>melhorar nome do campo indicando cidadão a listar materiais apresentados no local</t>
   </si>
   <si>
     <t>Tipo de ocupação:</t>
@@ -737,15 +734,9 @@
     <t>Dias da semana da ocorrência:</t>
   </si>
   <si>
-    <t>drop box</t>
-  </si>
-  <si>
     <t>Horário em que ocorre:</t>
   </si>
   <si>
-    <t>campo livre</t>
-  </si>
-  <si>
     <t>Acredito que o próprio serviço já fale por si só, não precisando da obrigatoriedade da descrição</t>
   </si>
   <si>
@@ -756,9 +747,6 @@
   </si>
   <si>
     <t>É quiosque de praia? :</t>
-  </si>
-  <si>
-    <t>o que isso muda no atendimento? precisa ser um campo extra?</t>
   </si>
   <si>
     <t>Descrição detalhada da ocorrência:</t>
@@ -784,10 +772,6 @@
   </si>
   <si>
     <t>pelo script os itens avaliados não faz sentido ter compplemento (chaminé, antena)</t>
-  </si>
-  <si>
-    <t>drop box
-Órgão precisa saber disso p atender?</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +990,9 @@
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1191,7 +1177,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Pedro Henrique Meireles Viana" id="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" providerId="google-sheets"/>
+  <x18tc:person displayName="Pedro Henrique Meireles Viana" id="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -1391,16 +1377,16 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A18" dT="2026-04-13T18:58:10.00" personId="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" id="{f5a66fda-0c81-42df-af30-4c66e2255bc0}" done="0">
+  <x18tc:threadedComment ref="A18" dT="2026-04-13T18:58:10.00" personId="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" id="{3e2ffa88-8395-46b4-a6ff-8043f985b458}" done="0">
     <x18tc:text xml:space="preserve">Revisitar o campo "Dados ou Documentos necessários".</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A35" dT="2026-04-13T17:29:15.00" personId="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" id="{2b894185-2081-4d23-aa1b-4055f8e1f2a8}" done="1">
+  <x18tc:threadedComment ref="A35" dT="2026-04-13T17:29:15.00" personId="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" id="{106fe65b-207a-4fef-bb5d-65c426ae0dfe}" done="1">
     <x18tc:text xml:space="preserve">Caso o campo "Informar se o obstáculo está fixado no chão" tenha como resposta "não", sugere-se que o campo "Informar se a calçada foi fechada com cancela, portão, grade ou guarita" seja fechado.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A18" dT="2026-04-13T17:24:02.00" personId="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" id="{99afa052-999d-44e4-8770-211425b04150}" done="1">
+  <x18tc:threadedComment ref="A18" dT="2026-04-13T17:24:02.00" personId="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" id="{cada2db6-c675-4d37-b110-ba5b0f389f52}" done="1">
     <x18tc:text xml:space="preserve">Revisitar o campo "Dados ou Documentos necessários".</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A26" dT="2026-04-13T18:57:51.00" personId="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" id="{da57aa93-8abe-4959-84c8-4bf38f451ac0}" done="0">
+  <x18tc:threadedComment ref="A26" dT="2026-04-13T18:57:51.00" personId="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" id="{9310f6d9-ace3-4304-81fe-60292bb798e5}" done="0">
     <x18tc:text xml:space="preserve">O script solicita a necessidade de informar o tipo de pavimento, porém no formulário não há campo que deixe claro o preenchimento dessa informação.</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1408,7 +1394,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A3" dT="2026-04-14T13:22:57.00" personId="{0b76e6ee-1d33-4e43-afc2-71b289ab47c2}" id="{4e9f8ac5-f033-44ea-b9dc-147610cecf1c}" done="0">
+  <x18tc:threadedComment ref="A3" dT="2026-04-14T13:22:57.00" personId="{4283a3a9-bec5-4c3f-b0d2-ddc43479db22}" id="{748f1715-cd33-4762-9a80-024903a734da}" done="0">
     <x18tc:text xml:space="preserve">Não existe campo para informações do acompanhante.</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -2153,7 +2139,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <tabColor rgb="FF9900FF"/>
+    <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
@@ -4032,7 +4018,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <tabColor rgb="FF9900FF"/>
+    <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
@@ -4246,10 +4232,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>207</v>
+        <v>8</v>
       </c>
       <c r="G7" s="50"/>
       <c r="H7" s="28"/>
@@ -4272,22 +4255,22 @@
     </row>
     <row r="8">
       <c r="A8" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>208</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>209</v>
       </c>
       <c r="G8" s="50"/>
       <c r="H8" s="29"/>
@@ -4310,7 +4293,7 @@
     </row>
     <row r="9">
       <c r="A9" s="48" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>8</v>
@@ -4319,12 +4302,11 @@
         <v>8</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="27"/>
+        <v>9</v>
+      </c>
       <c r="G9" s="50"/>
       <c r="H9" s="29"/>
       <c r="I9" s="29"/>
@@ -4358,7 +4340,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="50"/>
@@ -4382,7 +4364,7 @@
     </row>
     <row r="11">
       <c r="A11" s="48" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>8</v>
@@ -4396,9 +4378,7 @@
       <c r="E11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>212</v>
-      </c>
+      <c r="F11" s="8"/>
       <c r="G11" s="49"/>
       <c r="H11" s="29"/>
       <c r="I11" s="29"/>
@@ -4420,7 +4400,7 @@
     </row>
     <row r="12">
       <c r="A12" s="48" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>8</v>
@@ -4434,9 +4414,7 @@
       <c r="E12" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>214</v>
-      </c>
+      <c r="F12" s="8"/>
       <c r="G12" s="49"/>
       <c r="H12" s="29"/>
       <c r="I12" s="29"/>
@@ -4473,7 +4451,7 @@
         <v>9</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G13" s="49"/>
       <c r="H13" s="29"/>
@@ -4496,7 +4474,7 @@
     </row>
     <row r="14">
       <c r="A14" s="24" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="15">
@@ -4554,7 +4532,7 @@
       <c r="F17" s="27"/>
     </row>
     <row r="18">
-      <c r="A18" s="48" t="s">
+      <c r="A18" s="51" t="s">
         <v>159</v>
       </c>
       <c r="B18" s="7" t="s">
@@ -4564,14 +4542,12 @@
         <v>9</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>194</v>
-      </c>
+      <c r="F18" s="8"/>
     </row>
     <row r="19">
       <c r="A19" s="48" t="s">
@@ -4605,11 +4581,9 @@
         <v>8</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>207</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="F20" s="8"/>
     </row>
     <row r="21">
       <c r="A21" s="48" t="s">
@@ -4625,13 +4599,13 @@
         <v>8</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F21" s="8"/>
     </row>
     <row r="22">
       <c r="A22" s="48" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>8</v>
@@ -4649,7 +4623,7 @@
     </row>
     <row r="23">
       <c r="A23" s="48" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>8</v>
@@ -4658,18 +4632,16 @@
         <v>8</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>219</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="F23" s="8"/>
     </row>
     <row r="24">
       <c r="A24" s="48" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>8</v>
@@ -4684,7 +4656,7 @@
         <v>9</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25">
@@ -4704,7 +4676,7 @@
         <v>8</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -4726,7 +4698,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <tabColor rgb="FF9900FF"/>
+    <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
@@ -4792,7 +4764,7 @@
     </row>
     <row r="3">
       <c r="A3" s="24" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G3" s="24"/>
       <c r="H3" s="24"/>
@@ -4974,7 +4946,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" s="29"/>
       <c r="G8" s="50"/>
@@ -4998,7 +4970,7 @@
     </row>
     <row r="9">
       <c r="A9" s="48" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>8</v>
@@ -5043,13 +5015,13 @@
         <v>8</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="G10" s="49"/>
       <c r="H10" s="29"/>
@@ -5072,7 +5044,7 @@
     </row>
     <row r="11">
       <c r="A11" s="24" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12">
@@ -5140,13 +5112,13 @@
         <v>9</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>9</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16">
@@ -5163,13 +5135,13 @@
         <v>8</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" s="29"/>
     </row>
     <row r="17">
       <c r="A17" s="48" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>8</v>
@@ -5178,17 +5150,15 @@
         <v>9</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>228</v>
-      </c>
+      <c r="F17" s="7"/>
     </row>
     <row r="18">
-      <c r="A18" s="48" t="s">
+      <c r="A18" s="51" t="s">
         <v>166</v>
       </c>
       <c r="B18" s="7" t="s">
@@ -5201,10 +5171,10 @@
         <v>8</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -5301,16 +5271,11 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="18"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="s">
+    <row r="10">
+      <c r="A10" s="18" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="s">
+      <c r="B10" s="15" t="s">
         <v>39</v>
       </c>
     </row>
@@ -15017,7 +14982,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3"/>
+      <c r="A1" s="3">
+        <v>454.0</v>
+      </c>
       <c r="B1" s="4" t="s">
         <v>2</v>
       </c>
@@ -18542,6 +18509,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
+    <tabColor rgb="FFD9EAD3"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>

</xml_diff>